<commit_message>
chore: optimize bundle size with code splitting
</commit_message>
<xml_diff>
--- a/public/templates/DAFTAR AGENDA TUTOR.xlsx
+++ b/public/templates/DAFTAR AGENDA TUTOR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\web\production\E-learning\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE38427-8707-4176-B4B3-1DC8C08E384F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1A7B302-07B1-43FF-AA23-21B00ED6AAB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="390" windowWidth="29040" windowHeight="15930" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>YAYASAN MENUJU MAKMUR</t>
   </si>
@@ -161,6 +161,9 @@
   </si>
   <si>
     <t>NIP. ${nipTutor}</t>
+  </si>
+  <si>
+    <t>${mapel}</t>
   </si>
 </sst>
 </file>
@@ -823,7 +826,7 @@
     <xf numFmtId="0" fontId="30" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -873,48 +876,49 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="45">
     <cellStyle name="20% - Accent1" xfId="5" builtinId="30" customBuiltin="1"/>
@@ -1395,82 +1399,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
     </row>
     <row r="2" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
     </row>
     <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
     </row>
     <row r="5" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="24"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
     </row>
     <row r="7" spans="1:9" ht="7.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6"/>
@@ -1495,43 +1499,43 @@
       <c r="I8" s="6"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="22"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="24"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="8"/>
@@ -1545,10 +1549,10 @@
       <c r="I12" s="8"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="25"/>
+      <c r="B13" s="28"/>
       <c r="C13" s="9" t="s">
         <v>10</v>
       </c>
@@ -1586,37 +1590,37 @@
       <c r="I15" s="8"/>
     </row>
     <row r="16" spans="1:9" s="1" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D16" s="20" t="s">
+      <c r="D16" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E16" s="20" t="s">
+      <c r="E16" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="20" t="s">
+      <c r="F16" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="G16" s="20" t="s">
+      <c r="G16" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
     </row>
     <row r="17" spans="1:9" s="1" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="30"/>
-      <c r="B17" s="30"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
+      <c r="A17" s="21"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
       <c r="G17" s="10" t="s">
         <v>20</v>
       </c>
@@ -1660,10 +1664,10 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
-      <c r="H30" s="19" t="s">
+      <c r="H30" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="I30" s="19"/>
+      <c r="I30" s="32"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="15"/>
@@ -1673,19 +1677,18 @@
       <c r="E31" s="17"/>
       <c r="F31" s="17"/>
       <c r="G31" s="17"/>
-      <c r="H31" s="19" t="s">
+      <c r="H31" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="I31" s="19"/>
+      <c r="I31" s="32"/>
     </row>
     <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="15"/>
       <c r="B32" s="16"/>
       <c r="C32" s="16"/>
-      <c r="H32" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="I32" s="19"/>
+      <c r="H32" s="33" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="33" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="15"/>
@@ -1705,8 +1708,10 @@
       <c r="A35" s="15"/>
       <c r="B35" s="16"/>
       <c r="C35" s="16"/>
-      <c r="H35" s="18"/>
-      <c r="I35" s="18"/>
+      <c r="H35" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="I35" s="32"/>
     </row>
     <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="15"/>
@@ -1728,6 +1733,18 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A4:I4"/>
     <mergeCell ref="E16:E17"/>
     <mergeCell ref="D16:D17"/>
     <mergeCell ref="B16:B17"/>
@@ -1736,18 +1753,6 @@
     <mergeCell ref="C16:C17"/>
     <mergeCell ref="A10:I10"/>
     <mergeCell ref="G16:I16"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A9:I9"/>
-    <mergeCell ref="A11:I11"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="F16:F17"/>
   </mergeCells>
   <conditionalFormatting sqref="A18:I18">
     <cfRule type="expression" dxfId="0" priority="1">

</xml_diff>